<commit_message>
made a function to optimize unusedenzymesector intercept during parametrization and created unit tests
</commit_message>
<xml_diff>
--- a/tests/data/diagnostics_file_for_toy.xlsx
+++ b/tests/data/diagnostics_file_for_toy.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="39">
   <si>
     <t xml:space="preserve">Explanation for the test cases</t>
   </si>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t xml:space="preserve">TranslationalProteinSector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UnusedEnzymeSector</t>
   </si>
 </sst>
 </file>
@@ -267,7 +270,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:B5"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -315,7 +318,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.94140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.22"/>
@@ -610,7 +613,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.94140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.22"/>
@@ -905,7 +908,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.39"/>
@@ -942,8 +945,18 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+      <c r="A3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>-1E-006</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1E-005</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
added reversion of parametrization when solution is infeasible
</commit_message>
<xml_diff>
--- a/tests/data/diagnostics_file_for_toy.xlsx
+++ b/tests/data/diagnostics_file_for_toy.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="38">
   <si>
     <t xml:space="preserve">Explanation for the test cases</t>
   </si>
@@ -137,9 +137,6 @@
   </si>
   <si>
     <t xml:space="preserve">TranslationalProteinSector</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UnusedEnzymeSector</t>
   </si>
 </sst>
 </file>
@@ -270,7 +267,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:B5"/>
-  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -318,7 +315,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="8.94140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.22"/>
@@ -613,7 +610,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="8.94140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.22"/>
@@ -908,7 +905,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.39"/>
@@ -945,18 +942,8 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>-1E-006</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>1E-005</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
enabled changing of the sector parameters based on diagnostic file
</commit_message>
<xml_diff>
--- a/tests/data/diagnostics_file_for_toy.xlsx
+++ b/tests/data/diagnostics_file_for_toy.xlsx
@@ -267,7 +267,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:B5"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -315,7 +315,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.94140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.22"/>
@@ -610,7 +610,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.94140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.22"/>
@@ -905,7 +905,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.39"/>
@@ -932,10 +932,10 @@
         <v>36</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1E-005</v>
+        <v>1E-006</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1E-005</v>
+        <v>1E-006</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
most unit tests pass
</commit_message>
<xml_diff>
--- a/tests/data/diagnostics_file_for_toy.xlsx
+++ b/tests/data/diagnostics_file_for_toy.xlsx
@@ -267,7 +267,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:B5"/>
-  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -315,7 +315,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="8.94140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.95703125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.22"/>
@@ -610,7 +610,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="8.94140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.95703125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.22"/>
@@ -905,7 +905,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.39"/>
@@ -932,10 +932,10 @@
         <v>36</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1E-006</v>
+        <v>1E-005</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1E-006</v>
+        <v>1E-005</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>37</v>

</xml_diff>